<commit_message>
Add dependency for xls read support
</commit_message>
<xml_diff>
--- a/tests/test_core/dummy_data/aliases.xlsx
+++ b/tests/test_core/dummy_data/aliases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\crandall\Documents\ampworks\tests\test_core\dummy_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{57B0201F-7E1B-4A24-9FB4-EF2983615C51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA589FBF-5D62-4B95-B78A-B141CC33D6EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BFE1A89D-4FA1-48BA-B567-8E60ACB76DBC}"/>
   </bookViews>
@@ -28,9 +28,6 @@
     <t>amps_raw</t>
   </si>
   <si>
-    <t>volts_raw</t>
-  </si>
-  <si>
     <t>Meta</t>
   </si>
   <si>
@@ -38,6 +35,9 @@
   </si>
   <si>
     <t>b</t>
+  </si>
+  <si>
+    <t>Voltage (V)</t>
   </si>
 </sst>
 </file>
@@ -909,10 +909,10 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -926,7 +926,7 @@
         <v>3.1</v>
       </c>
       <c r="D2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -940,10 +940,16 @@
         <v>3.2</v>
       </c>
       <c r="D3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{95965d95-ecc0-4720-b759-1f33c42ed7da}" enabled="1" method="Standard" siteId="{a0f29d7e-28cd-4f54-8442-7885aee7c080}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>